<commit_message>
Add IFEEDER 2023 base check to vitamin D3 market-size model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBem8iwrXopPNAx2BvshQ4
</commit_message>
<xml_diff>
--- a/reports/Vitamin D3 market size model.xlsx
+++ b/reports/Vitamin D3 market size model.xlsx
@@ -21,12 +21,13 @@
     <definedName function="false" hidden="false" name="Base2020" vbProcedure="false">Inputs!$C$4</definedName>
     <definedName function="false" hidden="false" name="Base2020_H" vbProcedure="false">Inputs!$E$4</definedName>
     <definedName function="false" hidden="false" name="Base2020_L" vbProcedure="false">Inputs!$D$4</definedName>
-    <definedName function="false" hidden="false" name="Base2022User" vbProcedure="false">Inputs!$C$19</definedName>
+    <definedName function="false" hidden="false" name="Base2022User" vbProcedure="false">Inputs!$C$25</definedName>
     <definedName function="false" hidden="false" name="Feed2020Mt" vbProcedure="false">'Feed index'!$B$5</definedName>
     <definedName function="false" hidden="false" name="FeedG2026" vbProcedure="false">Inputs!$C$7</definedName>
     <definedName function="false" hidden="false" name="FeedG2026_H" vbProcedure="false">Inputs!$E$7</definedName>
     <definedName function="false" hidden="false" name="FeedG2026_L" vbProcedure="false">Inputs!$D$7</definedName>
     <definedName function="false" hidden="false" name="FeedIdx2022" vbProcedure="false">'Feed index'!$D$7</definedName>
+    <definedName function="false" hidden="false" name="FeedIdx2023" vbProcedure="false">'Feed index'!$D$8</definedName>
     <definedName function="false" hidden="false" name="FeedIdx2025" vbProcedure="false">'Feed index'!$D$10</definedName>
     <definedName function="false" hidden="false" name="FeedP2020" vbProcedure="false">Inputs!$C$11</definedName>
     <definedName function="false" hidden="false" name="FeedP2020_H" vbProcedure="false">Inputs!$E$11</definedName>
@@ -40,15 +41,18 @@
     <definedName function="false" hidden="false" name="FeedP2026" vbProcedure="false">Inputs!$C$14</definedName>
     <definedName function="false" hidden="false" name="FeedP2026_H" vbProcedure="false">Inputs!$E$14</definedName>
     <definedName function="false" hidden="false" name="FeedP2026_L" vbProcedure="false">Inputs!$D$14</definedName>
-    <definedName function="false" hidden="false" name="FX_INR" vbProcedure="false">Inputs!$C$22</definedName>
-    <definedName function="false" hidden="false" name="FX_RMB" vbProcedure="false">Inputs!$C$20</definedName>
-    <definedName function="false" hidden="false" name="FX_RMB22" vbProcedure="false">Inputs!$C$21</definedName>
+    <definedName function="false" hidden="false" name="FX_INR" vbProcedure="false">Inputs!$C$28</definedName>
+    <definedName function="false" hidden="false" name="FX_RMB" vbProcedure="false">Inputs!$C$26</definedName>
+    <definedName function="false" hidden="false" name="FX_RMB22" vbProcedure="false">Inputs!$C$27</definedName>
     <definedName function="false" hidden="false" name="HumanShare" vbProcedure="false">Inputs!$C$6</definedName>
     <definedName function="false" hidden="false" name="HumanShare_H" vbProcedure="false">Inputs!$E$6</definedName>
     <definedName function="false" hidden="false" name="HumanShare_L" vbProcedure="false">Inputs!$D$6</definedName>
     <definedName function="false" hidden="false" name="HumIdx2022" vbProcedure="false">Inputs!$C$8</definedName>
     <definedName function="false" hidden="false" name="HumIdx2022_H" vbProcedure="false">Inputs!$E$8</definedName>
     <definedName function="false" hidden="false" name="HumIdx2022_L" vbProcedure="false">Inputs!$D$8</definedName>
+    <definedName function="false" hidden="false" name="HumIdx2023" vbProcedure="false">Inputs!$C$19</definedName>
+    <definedName function="false" hidden="false" name="HumIdx2023_H" vbProcedure="false">Inputs!$E$19</definedName>
+    <definedName function="false" hidden="false" name="HumIdx2023_L" vbProcedure="false">Inputs!$D$19</definedName>
     <definedName function="false" hidden="false" name="HumIdx2025" vbProcedure="false">Inputs!$C$9</definedName>
     <definedName function="false" hidden="false" name="HumIdx2025_H" vbProcedure="false">Inputs!$E$9</definedName>
     <definedName function="false" hidden="false" name="HumIdx2025_L" vbProcedure="false">Inputs!$D$9</definedName>
@@ -67,6 +71,11 @@
     <definedName function="false" hidden="false" name="HumP2026" vbProcedure="false">Inputs!$C$18</definedName>
     <definedName function="false" hidden="false" name="HumP2026_H" vbProcedure="false">Inputs!$E$18</definedName>
     <definedName function="false" hidden="false" name="HumP2026_L" vbProcedure="false">Inputs!$D$18</definedName>
+    <definedName function="false" hidden="false" name="IF_BasisA" vbProcedure="false">Inputs!$C$23</definedName>
+    <definedName function="false" hidden="false" name="IF_BasisB" vbProcedure="false">Inputs!$C$24</definedName>
+    <definedName function="false" hidden="false" name="IF_Cap" vbProcedure="false">Inputs!$C$22</definedName>
+    <definedName function="false" hidden="false" name="IF_Demand" vbProcedure="false">Inputs!$C$21</definedName>
+    <definedName function="false" hidden="false" name="IF_Supply" vbProcedure="false">Inputs!$C$20</definedName>
     <definedName function="false" hidden="false" name="Potency" vbProcedure="false">Inputs!$C$5</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -79,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="476">
   <si>
     <t xml:space="preserve">Vitamin D3 global market size: extrapolation model (2020/2022 base to 2026E)</t>
   </si>
@@ -151,6 +160,9 @@
   </si>
   <si>
     <t xml:space="preserve">2025 value, USD m (for comparison)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026E value from IFEEDER 2023 base, USD m (500K / 1 MIU readings)</t>
   </si>
   <si>
     <t xml:space="preserve">Inputs: edit blue cells only</t>
@@ -550,6 +562,93 @@
     <t xml:space="preserve">Analyst assumption: flat on 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">D0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human volume index 2023 (2020 = 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst assumption: Fermenta filed human volumes give CY2023/CY2020 = 0.73 (FY23 -30%, FY24 -18%); CARE Nov 2023: channel 'saddled with surplus stocks'; dsm-firmenich FY2023 HNC volumes -6% ('persistent destocking'). End-consumption fell less than Fermenta's sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used only in the IFEEDER 2023 base check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER 2023 global D3 supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT (basis unstated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision Innovation Solutions &amp; Lobo Consulting Solutions for IFEEDER (AFIA research foundation), 'Strategic Assessment on Impact of Vitamin and Amino Acid Supply Chain Disruptions on U.S. Food Security', section 3.3.3: 'estimate global vitamin D3 supply for 2023 at 3,640 MT'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Institutional study (consultant estimates)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No IU/g potency basis is given anywhere in the section. p.2 table labels 3,639 as capacity (inconsistent).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER 2023 global D3 demand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision Innovation Solutions &amp; Lobo Consulting Solutions for IFEEDER (AFIA research foundation), 'Strategic Assessment on Impact of Vitamin and Amino Acid Supply Chain Disruptions on U.S. Food Security', section 3.3.3: 'global demand at approximately 3,755 MT'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER 2023 global D3 capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision Innovation Solutions &amp; Lobo Consulting Solutions for IFEEDER (AFIA research foundation), 'Strategic Assessment on Impact of Vitamin and Amino Acid Supply Chain Disruptions on U.S. Food Security', section 3.3.3: capacity 'about 19,000 MT' (corroborated by 'multiple industry sources'); flat to June 2025; utilisation 20%; China ~93%, India 5%, EU 3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p.23, Fig. 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity/demand of ~5x matches FEFAC's 'five times demand' (2025 factsheet).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading A: IU/g basis of IFEEDER tonnes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IU/g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst assumption: industry convention for feed-grade tonnage (D3-500)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading B: IU/g basis of IFEEDER tonnes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst assumption: D3 1.0 MIU/g (oil) convention</t>
+  </si>
+  <si>
     <t xml:space="preserve">G1</t>
   </si>
   <si>
@@ -838,6 +937,87 @@
     <t xml:space="preserve">Interpretation: API-equivalent human value prices all human volume at crystalline USD/kg; formulated forms (oils, CWS beadlets, spray-dried D3 100) sell at several times that per IU, so an 'as-sold' human market is larger (see Cross-checks). For an API maker such as Symbiotec, the API-equivalent pool is the relevant addressable market.</t>
   </si>
   <si>
+    <t xml:space="preserve">2023 IFEEDER base check (English public source; potency basis unstated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading A: 500,000 IU/g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading B: 1,000,000 IU/g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER 2023 supply, MT as stated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs J1 (p.23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumed potency, IU/g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs J4/J5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023 supply, t D3-500 equivalent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT x IU/g ÷ 500,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023 supply, t pure D3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model's own 2023 volume (2020 base), t D3-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boyar 2020 base rolled to 2023 with the same indices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER as % of model 2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human share of 2023 volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From the model path</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed multiplier 2023 -&gt; 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human multiplier 2023 -&gt; 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human index ratio (2023 destock trough)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026E volume from IFEEDER base, t D3-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026E value from IFEEDER base, USD m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same 2026 prices as the main model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs 2020-base 2026E value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER capacity, t pure D3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare ~184 t pure in Chinese broker capacity tables (14,740 t D3-500)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IFEEDER capacity ÷ demand (x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis-independent; FEFAC 2025 says 'five times'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading: on 500,000 IU/g the IFEEDER supply is ~45 t pure, about 40% below the Boyar-based 2023 path and half the ~100 t pure in dsm-firmenich authors' OPRD paper; on 1,000,000 IU/g it is ~91 t pure (consistent with both), but its capacity would then be ~475 t pure, ~2.6x Chinese capacity tables. No single basis reconciles all three IFEEDER numbers, so it brackets the base case rather than replacing it.</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026E total value (USD m): feed-grade price x human share</t>
   </si>
   <si>
@@ -1006,7 +1186,7 @@
     <t xml:space="preserve">Quote read via search index (publisher blocked); year not stated.</t>
   </si>
   <si>
-    <t xml:space="preserve">Supply 3,640 MT; demand ~3,755 MT; capacity ~19,000 MT</t>
+    <t xml:space="preserve">Supply 3,640 MT; demand ~3,755 MT; capacity ~19,000 MT; China ~93% of capacity</t>
   </si>
   <si>
     <t xml:space="preserve">Supply/demand</t>
@@ -1015,19 +1195,13 @@
     <t xml:space="preserve">IFEEDER (AFIA foundation) / DIS &amp; LCS, Strategic Assessment on Vitamin and Amino Acid Supply Chain Disruptions</t>
   </si>
   <si>
-    <t xml:space="preserve">p.23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee</t>
-  </si>
-  <si>
     <t xml:space="preserve">Institutional study</t>
   </si>
   <si>
-    <t xml:space="preserve">Basis unstated and internally inconsistent (p.2 labels 3,639 as capacity); low confidence.</t>
+    <t xml:space="preserve">Check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis unstated; see Model rows 38-56 for both readings. p.2 table labels 3,639 as capacity.</t>
   </si>
   <si>
     <t xml:space="preserve">10,308 t (feed 8,189 t)</t>
@@ -1178,9 +1352,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cross-checks against company disclosures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check</t>
   </si>
   <si>
     <t xml:space="preserve">Garden 2025: implied market from revenue/share</t>
@@ -1455,7 +1626,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
@@ -1468,7 +1639,8 @@
     <numFmt numFmtId="173" formatCode="0.000"/>
     <numFmt numFmtId="174" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="175" formatCode="0.0\x"/>
-    <numFmt numFmtId="176" formatCode="#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="0%;\(0%\);\-"/>
+    <numFmt numFmtId="177" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1641,7 +1813,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1798,6 +1970,14 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1826,7 +2006,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2086,7 +2266,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -2219,6 +2399,15 @@
       <c r="B18" s="5" t="n">
         <f aca="false">Model!D22</f>
         <v>212.443111513341</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="7" t="str">
+        <f aca="false">TEXT(Model!B51,"#,##0")&amp;" / "&amp;TEXT(Model!C51,"#,##0")</f>
+        <v>94 / 187</v>
       </c>
     </row>
   </sheetData>
@@ -2237,7 +2426,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2255,53 +2444,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="47.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>6250</v>
@@ -2313,33 +2502,33 @@
         <v>6500</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>80</v>
@@ -2347,31 +2536,31 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6" s="15" t="n">
         <v>0.2</v>
@@ -2383,33 +2572,33 @@
         <v>0.3</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C7" s="15" t="n">
         <v>0.015</v>
@@ -2421,31 +2610,31 @@
         <v>0.02</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>0.95</v>
@@ -2457,31 +2646,31 @@
         <v>1</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" s="14" t="n">
         <v>1.13</v>
@@ -2493,31 +2682,31 @@
         <v>1.2</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>1.15</v>
@@ -2529,29 +2718,29 @@
         <v>1.28</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>26</v>
@@ -2563,33 +2752,33 @@
         <v>30</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C12" s="18" t="n">
         <v>11.5</v>
@@ -2601,33 +2790,33 @@
         <v>13</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C13" s="11" t="n">
         <v>32</v>
@@ -2639,29 +2828,29 @@
         <v>40</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>21</v>
@@ -2673,31 +2862,31 @@
         <v>25</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C15" s="11" t="n">
         <v>2200</v>
@@ -2709,29 +2898,29 @@
         <v>3300</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C16" s="11" t="n">
         <v>2390</v>
@@ -2743,29 +2932,29 @@
         <v>3300</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C17" s="11" t="n">
         <v>2420</v>
@@ -2777,29 +2966,29 @@
         <v>3300</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>2420</v>
@@ -2811,129 +3000,317 @@
         <v>3300</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I18" s="3"/>
       <c r="J18" s="12"/>
       <c r="K18" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L18" s="12"/>
     </row>
-    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
+        <v>141</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F19" s="3" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="H19" s="3"/>
+        <v>142</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>143</v>
+      </c>
       <c r="I19" s="3"/>
-      <c r="J19" s="12"/>
+      <c r="J19" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="K19" s="3" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C20" s="18" t="n">
-        <v>7.2</v>
+        <v>146</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>3640</v>
       </c>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="12"/>
+        <v>148</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>151</v>
+      </c>
       <c r="K20" s="3" t="s">
-        <v>69</v>
+        <v>152</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="18" t="n">
-        <v>6.7</v>
+        <v>155</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>3755</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
       <c r="F21" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G21" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J21" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="12"/>
       <c r="K21" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="L21" s="12" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L21" s="12"/>
+    </row>
+    <row r="22" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>88</v>
+        <v>19000</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
       <c r="F22" s="3" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="12"/>
+        <v>159</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>151</v>
+      </c>
       <c r="K22" s="3" t="s">
-        <v>69</v>
+        <v>152</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>148</v>
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="L23" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="L24" s="12"/>
+    </row>
+    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C25" s="10"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="L25" s="12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="L27" s="12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>88</v>
+      </c>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2952,6 +3329,10 @@
     <hyperlink ref="J15" r:id="rId12" display="https://www.bseindia.com/xml-data/corpfiling/AttachHis/23445550-d343-4c2e-98b8-ed6d83f24557.pdf"/>
     <hyperlink ref="J16" r:id="rId13" display="https://tradestat.commerce.gov.in/eidb/commodity_wise_all_countries_export"/>
     <hyperlink ref="J17" r:id="rId14" display="https://tradestat.commerce.gov.in/eidb/commodity_wise_all_countries_export"/>
+    <hyperlink ref="J19" r:id="rId15" display="https://www.careratings.com/upload/CompanyFiles/PR/202311131111_Fermenta_Biotech_Limited.pdf"/>
+    <hyperlink ref="J20" r:id="rId16" display="https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee"/>
+    <hyperlink ref="J21" r:id="rId17" display="https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee"/>
+    <hyperlink ref="J22" r:id="rId18" display="https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2982,40 +3363,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>1187.7</v>
@@ -3027,18 +3408,18 @@
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>166</v>
+        <v>196</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1235</v>
@@ -3051,18 +3432,18 @@
         <v>1.023</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>169</v>
+        <v>199</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>1266</v>
@@ -3075,18 +3456,18 @@
         <v>1.0187034</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>1290</v>
@@ -3099,18 +3480,18 @@
         <v>1.01860152966</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>175</v>
+        <v>205</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>176</v>
+        <v>206</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>167</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>177</v>
+        <v>207</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>1396</v>
@@ -3123,18 +3504,18 @@
         <v>1.03082474801592</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>179</v>
+        <v>209</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>180</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>1440</v>
@@ -3147,18 +3528,18 @@
         <v>1.06071866570838</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>182</v>
+        <v>212</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>183</v>
+        <v>213</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>180</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>184</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -3185,7 +3566,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -3195,32 +3576,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>187</v>
+        <v>217</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>188</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>189</v>
+        <v>219</v>
       </c>
       <c r="B4" s="25"/>
       <c r="C4" s="25"/>
@@ -3230,7 +3611,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="B5" s="26" t="n">
         <v>1</v>
@@ -3248,12 +3629,12 @@
         <v>1.07662944569401</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>191</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>192</v>
+        <v>222</v>
       </c>
       <c r="B6" s="26" t="n">
         <v>1</v>
@@ -3271,12 +3652,12 @@
         <v>1.15</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>193</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>194</v>
+        <v>224</v>
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">Base2020*(1-HumanShare)*B5</f>
@@ -3295,12 +3676,12 @@
         <v>5383.14722847004</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>195</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>196</v>
+        <v>226</v>
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">Base2020*HumanShare*B6</f>
@@ -3319,12 +3700,12 @@
         <v>1437.5</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>197</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>198</v>
+        <v>228</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">B7+B8</f>
@@ -3346,7 +3727,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>199</v>
+        <v>229</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">B9/Potency</f>
@@ -3365,12 +3746,12 @@
         <v>85.2580903558755</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>200</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>201</v>
+        <v>231</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">B8/Potency</f>
@@ -3392,7 +3773,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>202</v>
+        <v>232</v>
       </c>
       <c r="B12" s="31" t="n">
         <f aca="false">B9/$B$9-1</f>
@@ -3414,7 +3795,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>203</v>
+        <v>233</v>
       </c>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
@@ -3424,7 +3805,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>204</v>
+        <v>234</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">FeedP2020</f>
@@ -3443,12 +3824,12 @@
         <v>21</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>205</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>206</v>
+        <v>236</v>
       </c>
       <c r="B16" s="33" t="n">
         <f aca="false">HumP2020</f>
@@ -3467,12 +3848,12 @@
         <v>2420</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>207</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>208</v>
+        <v>238</v>
       </c>
       <c r="B17" s="34" t="n">
         <f aca="false">B16/Potency/B15</f>
@@ -3491,12 +3872,12 @@
         <v>1.44047619047619</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>209</v>
+        <v>239</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
@@ -3506,7 +3887,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>211</v>
+        <v>241</v>
       </c>
       <c r="B20" s="28" t="n">
         <f aca="false">B7*B15/1000</f>
@@ -3525,12 +3906,12 @@
         <v>113.046091797871</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>213</v>
+        <v>243</v>
       </c>
       <c r="B21" s="28" t="n">
         <f aca="false">B11*B16/1000</f>
@@ -3549,12 +3930,12 @@
         <v>43.484375</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>214</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>215</v>
+        <v>245</v>
       </c>
       <c r="B22" s="29" t="n">
         <f aca="false">B20+B21</f>
@@ -3576,7 +3957,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>216</v>
+        <v>246</v>
       </c>
       <c r="B23" s="35" t="n">
         <f aca="false">IF(B22=0,0,B20/B22)</f>
@@ -3598,7 +3979,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>217</v>
+        <v>247</v>
       </c>
       <c r="B24" s="28" t="n">
         <f aca="false">B7*FeedP2020_L/1000+B11*HumP2020_L/1000</f>
@@ -3617,12 +3998,12 @@
         <v>122.060377883991</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>218</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="B25" s="28" t="n">
         <f aca="false">B7*FeedP2020_H/1000+B11*HumP2020_H/1000</f>
@@ -3641,65 +4022,65 @@
         <v>193.875555711751</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="36" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>222</v>
+        <v>252</v>
       </c>
       <c r="B28" s="28" t="n">
         <f aca="false">IF(ISNUMBER(Base2022User),Base2022User,C9)</f>
         <v>6281.017</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>223</v>
+        <v>253</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>224</v>
+        <v>254</v>
       </c>
       <c r="B29" s="37" t="n">
         <f aca="false">C8/C9</f>
         <v>0.189061739524029</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>225</v>
+        <v>255</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>226</v>
+        <v>256</v>
       </c>
       <c r="B30" s="26" t="n">
         <f aca="false">E5/C5</f>
         <v>1.056862523178</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>227</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>228</v>
+        <v>258</v>
       </c>
       <c r="B31" s="26" t="n">
         <f aca="false">E6/C6</f>
         <v>1.21052631578947</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>229</v>
+        <v>259</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>230</v>
+        <v>260</v>
       </c>
       <c r="B32" s="28" t="n">
         <f aca="false">B28*(1-B29)*B30+B28*B29*B31</f>
@@ -3709,7 +4090,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="B33" s="28" t="n">
         <f aca="false">B28*(1-B29)*B30*FeedP2026/1000+B28*B29*B31/Potency*HumP2026/1000</f>
@@ -3719,19 +4100,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>232</v>
+        <v>262</v>
       </c>
       <c r="B34" s="31" t="n">
         <f aca="false">IF(E22=0,0,B33/E22-1)</f>
         <v>0</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>233</v>
+        <v>263</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="38" t="s">
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="B36" s="38"/>
       <c r="C36" s="38"/>
@@ -3739,9 +4120,261 @@
       <c r="E36" s="38"/>
       <c r="F36" s="38"/>
     </row>
+    <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="B38" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="C38" s="39" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B40" s="33" t="n">
+        <f aca="false">IF_Supply</f>
+        <v>3640</v>
+      </c>
+      <c r="C40" s="33" t="n">
+        <f aca="false">IF_Supply</f>
+        <v>3640</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B41" s="33" t="n">
+        <f aca="false">IF_BasisA</f>
+        <v>500000</v>
+      </c>
+      <c r="C41" s="33" t="n">
+        <f aca="false">IF_BasisB</f>
+        <v>1000000</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="B42" s="28" t="n">
+        <f aca="false">B40*B41/500000</f>
+        <v>3640</v>
+      </c>
+      <c r="C42" s="28" t="n">
+        <f aca="false">C40*C41/500000</f>
+        <v>7280</v>
+      </c>
+      <c r="F42" s="19" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B43" s="30" t="n">
+        <f aca="false">B42/Potency</f>
+        <v>45.5</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <f aca="false">C42/Potency</f>
+        <v>91</v>
+      </c>
+      <c r="F43" s="19"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B44" s="28" t="n">
+        <f aca="false">Base2020*(1-HumanShare)*FeedIdx2023+Base2020*HumanShare*HumIdx2023</f>
+        <v>6093.0076483</v>
+      </c>
+      <c r="C44" s="28" t="n">
+        <f aca="false">Base2020*(1-HumanShare)*FeedIdx2023+Base2020*HumanShare*HumIdx2023</f>
+        <v>6093.0076483</v>
+      </c>
+      <c r="F44" s="19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B45" s="35" t="n">
+        <f aca="false">IF(B44=0,0,B42/B44)</f>
+        <v>0.597406110431453</v>
+      </c>
+      <c r="C45" s="35" t="n">
+        <f aca="false">IF(C44=0,0,C42/C44)</f>
+        <v>1.19481222086291</v>
+      </c>
+      <c r="F45" s="19"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B46" s="37" t="n">
+        <f aca="false">Base2020*HumanShare*HumIdx2023/B44</f>
+        <v>0.164122557810839</v>
+      </c>
+      <c r="C46" s="37" t="n">
+        <f aca="false">Base2020*HumanShare*HumIdx2023/C44</f>
+        <v>0.164122557810839</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="B47" s="26" t="n">
+        <f aca="false">$E$5/FeedIdx2023</f>
+        <v>1.05696822</v>
+      </c>
+      <c r="C47" s="26" t="n">
+        <f aca="false">$E$5/FeedIdx2023</f>
+        <v>1.05696822</v>
+      </c>
+      <c r="F47" s="19" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B48" s="26" t="n">
+        <f aca="false">HumIdx2026/HumIdx2023</f>
+        <v>1.4375</v>
+      </c>
+      <c r="C48" s="26" t="n">
+        <f aca="false">HumIdx2026/HumIdx2023</f>
+        <v>1.4375</v>
+      </c>
+      <c r="F48" s="19" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B49" s="28" t="n">
+        <f aca="false">B42*((1-B46)*B47+B46*B48)</f>
+        <v>4074.69633138536</v>
+      </c>
+      <c r="C49" s="28" t="n">
+        <f aca="false">C42*((1-C46)*C47+C46*C48)</f>
+        <v>8149.39266277071</v>
+      </c>
+      <c r="F49" s="19"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B50" s="30" t="n">
+        <f aca="false">B49/Potency</f>
+        <v>50.933704142317</v>
+      </c>
+      <c r="C50" s="30" t="n">
+        <f aca="false">C49/Potency</f>
+        <v>101.867408284634</v>
+      </c>
+      <c r="F50" s="19"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B51" s="28" t="n">
+        <f aca="false">B42*(1-B46)*B47*FeedP2026/1000+B42*B46*B48/Potency*HumP2026/1000</f>
+        <v>93.5122573337357</v>
+      </c>
+      <c r="C51" s="28" t="n">
+        <f aca="false">C42*(1-C46)*C47*FeedP2026/1000+C42*C46*C48/Potency*HumP2026/1000</f>
+        <v>187.024514667471</v>
+      </c>
+      <c r="F51" s="19" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B52" s="40" t="n">
+        <f aca="false">IF($E$22=0,0,B51/$E$22-1)</f>
+        <v>-0.402593889568547</v>
+      </c>
+      <c r="C52" s="40" t="n">
+        <f aca="false">IF($E$22=0,0,C51/$E$22-1)</f>
+        <v>0.194812220862907</v>
+      </c>
+      <c r="F52" s="19"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B53" s="28" t="n">
+        <f aca="false">IF_Cap*B41/500000/Potency</f>
+        <v>237.5</v>
+      </c>
+      <c r="C53" s="28" t="n">
+        <f aca="false">IF_Cap*C41/500000/Potency</f>
+        <v>475</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B54" s="34" t="n">
+        <f aca="false">IF_Cap/IF_Demand</f>
+        <v>5.05992010652463</v>
+      </c>
+      <c r="C54" s="34" t="n">
+        <f aca="false">IF_Cap/IF_Demand</f>
+        <v>5.05992010652463</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="38" t="s">
+        <v>291</v>
+      </c>
+      <c r="B56" s="38"/>
+      <c r="C56" s="38"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A56:F56"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3767,36 +4400,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>236</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="s">
-        <v>237</v>
-      </c>
-      <c r="B4" s="40" t="n">
+      <c r="A4" s="41" t="s">
+        <v>294</v>
+      </c>
+      <c r="B4" s="42" t="n">
         <v>0.11</v>
       </c>
-      <c r="C4" s="40" t="n">
+      <c r="C4" s="42" t="n">
         <v>0.15</v>
       </c>
-      <c r="D4" s="40" t="n">
+      <c r="D4" s="42" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="40" t="n">
+      <c r="E4" s="42" t="n">
         <v>0.25</v>
       </c>
-      <c r="F4" s="40" t="n">
+      <c r="F4" s="42" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="41" t="n">
+      <c r="A5" s="43" t="n">
         <v>15</v>
       </c>
       <c r="B5" s="28" t="n">
@@ -3821,7 +4454,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="41" t="n">
+      <c r="A6" s="43" t="n">
         <v>17</v>
       </c>
       <c r="B6" s="28" t="n">
@@ -3846,7 +4479,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="41" t="n">
+      <c r="A7" s="43" t="n">
         <v>19</v>
       </c>
       <c r="B7" s="28" t="n">
@@ -3871,7 +4504,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="41" t="n">
+      <c r="A8" s="43" t="n">
         <v>21</v>
       </c>
       <c r="B8" s="28" t="n">
@@ -3896,7 +4529,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="41" t="n">
+      <c r="A9" s="43" t="n">
         <v>23</v>
       </c>
       <c r="B9" s="28" t="n">
@@ -3921,7 +4554,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="41" t="n">
+      <c r="A10" s="43" t="n">
         <v>25</v>
       </c>
       <c r="B10" s="28" t="n">
@@ -3946,7 +4579,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="41" t="n">
+      <c r="A11" s="43" t="n">
         <v>30</v>
       </c>
       <c r="B11" s="28" t="n">
@@ -3971,7 +4604,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="41" t="n">
+      <c r="A12" s="43" t="n">
         <v>35</v>
       </c>
       <c r="B12" s="28" t="n">
@@ -3997,7 +4630,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>238</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -4036,609 +4669,609 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>239</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>240</v>
+        <v>297</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>241</v>
+        <v>298</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>242</v>
+        <v>299</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>243</v>
+        <v>300</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>244</v>
+        <v>301</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>245</v>
+        <v>302</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>246</v>
+        <v>303</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>247</v>
+        <v>304</v>
       </c>
       <c r="I3" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="K3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>248</v>
+        <v>305</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>249</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>250</v>
+        <v>307</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>251</v>
+        <v>308</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E4" s="42" t="n">
+        <v>309</v>
+      </c>
+      <c r="E4" s="44" t="n">
         <v>6250</v>
       </c>
-      <c r="F4" s="43" t="n">
+      <c r="F4" s="45" t="n">
         <f aca="false">E4/Potency</f>
         <v>78.125</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>253</v>
+        <v>310</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>254</v>
+        <v>311</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>256</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>257</v>
+        <v>314</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>258</v>
+        <v>315</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E5" s="42" t="n">
+        <v>309</v>
+      </c>
+      <c r="E5" s="44" t="n">
         <v>14600</v>
       </c>
-      <c r="F5" s="43" t="n">
+      <c r="F5" s="45" t="n">
         <f aca="false">E5/Potency</f>
         <v>182.5</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>253</v>
+        <v>310</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>259</v>
+        <v>316</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>255</v>
+        <v>312</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>261</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>262</v>
+        <v>319</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>263</v>
+        <v>320</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="E6" s="42" t="n">
+        <v>321</v>
+      </c>
+      <c r="E6" s="44" t="n">
         <v>7500</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="45" t="n">
         <f aca="false">E6/Potency</f>
         <v>93.75</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>266</v>
+        <v>323</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3" t="s">
-        <v>267</v>
+        <v>324</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>269</v>
+        <v>326</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>270</v>
+        <v>327</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>271</v>
+        <v>328</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>272</v>
+        <v>329</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>273</v>
+        <v>330</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>274</v>
+        <v>331</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="E7" s="42" t="n">
+        <v>332</v>
+      </c>
+      <c r="E7" s="44" t="n">
         <v>11000</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="45" t="n">
         <f aca="false">E7/Potency</f>
         <v>137.5</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>276</v>
+        <v>333</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>277</v>
+        <v>334</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>278</v>
+        <v>335</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>279</v>
+        <v>336</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>280</v>
+        <v>337</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>270</v>
+        <v>327</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>281</v>
+        <v>338</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>282</v>
+        <v>339</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>283</v>
+        <v>340</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="E8" s="42" t="n">
+        <v>342</v>
+      </c>
+      <c r="E8" s="44" t="n">
         <v>8000</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="45" t="n">
         <f aca="false">E8/Potency</f>
         <v>100</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>286</v>
+        <v>343</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>287</v>
+        <v>344</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>288</v>
+        <v>345</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>289</v>
+        <v>346</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>270</v>
+        <v>327</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>290</v>
+        <v>347</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>291</v>
+        <v>348</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>292</v>
+        <v>349</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="E9" s="42" t="n">
+        <v>321</v>
+      </c>
+      <c r="E9" s="44" t="n">
         <v>3640</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="45" t="n">
         <f aca="false">E9/Potency</f>
         <v>45.5</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>293</v>
+        <v>350</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>294</v>
+        <v>150</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>295</v>
+        <v>149</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>296</v>
+        <v>151</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>297</v>
+        <v>351</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>260</v>
+        <v>352</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>298</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>300</v>
+        <v>355</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E10" s="42" t="n">
+        <v>309</v>
+      </c>
+      <c r="E10" s="44" t="n">
         <v>10308</v>
       </c>
-      <c r="F10" s="43" t="n">
+      <c r="F10" s="45" t="n">
         <f aca="false">E10/Potency</f>
         <v>128.85</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>253</v>
+        <v>310</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>302</v>
+        <v>357</v>
       </c>
       <c r="K10" s="12"/>
       <c r="L10" s="3" t="s">
-        <v>303</v>
+        <v>358</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>305</v>
+        <v>360</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>306</v>
+        <v>361</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E11" s="42" t="n">
+        <v>309</v>
+      </c>
+      <c r="E11" s="44" t="n">
         <v>14793</v>
       </c>
-      <c r="F11" s="43" t="n">
+      <c r="F11" s="45" t="n">
         <f aca="false">E11/Potency</f>
         <v>184.9125</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>253</v>
+        <v>310</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>308</v>
+        <v>363</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>309</v>
+        <v>364</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N11" s="12" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>311</v>
+        <v>366</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>312</v>
+        <v>367</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>313</v>
+        <v>368</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E12" s="42" t="n">
+        <v>309</v>
+      </c>
+      <c r="E12" s="44" t="n">
         <v>6750</v>
       </c>
-      <c r="F12" s="43" t="n">
+      <c r="F12" s="45" t="n">
         <f aca="false">E12/Potency</f>
         <v>84.375</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>314</v>
+        <v>369</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>315</v>
+        <v>370</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>316</v>
+        <v>371</v>
       </c>
       <c r="K12" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="M12" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="L12" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>260</v>
-      </c>
       <c r="N12" s="12" t="s">
-        <v>319</v>
+        <v>374</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>321</v>
+        <v>376</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E13" s="44" t="n">
+        <v>309</v>
+      </c>
+      <c r="E13" s="46" t="n">
         <f aca="false">Model!C9</f>
         <v>6281.017</v>
       </c>
-      <c r="F13" s="43" t="n">
+      <c r="F13" s="45" t="n">
         <f aca="false">E13/Potency</f>
         <v>78.5127125</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>323</v>
+        <v>378</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="12"/>
       <c r="L13" s="3" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
       <c r="N13" s="12" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>326</v>
+        <v>381</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="E14" s="44"/>
+        <v>383</v>
+      </c>
+      <c r="E14" s="46"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>329</v>
+        <v>384</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3" t="s">
-        <v>267</v>
+        <v>324</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>330</v>
+        <v>385</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>331</v>
+        <v>386</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N14" s="12" t="s">
-        <v>332</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>333</v>
+        <v>388</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="E15" s="44"/>
+        <v>383</v>
+      </c>
+      <c r="E15" s="46"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>334</v>
+        <v>389</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3" t="s">
-        <v>335</v>
+        <v>390</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>336</v>
+        <v>391</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>331</v>
+        <v>386</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N15" s="12" t="s">
-        <v>337</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>338</v>
+        <v>393</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>339</v>
+        <v>394</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="E16" s="44"/>
+        <v>395</v>
+      </c>
+      <c r="E16" s="46"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3" t="s">
-        <v>265</v>
+        <v>322</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>341</v>
+        <v>396</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>342</v>
+        <v>397</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>343</v>
+        <v>398</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>344</v>
+        <v>399</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>345</v>
+        <v>400</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>346</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>347</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -4683,369 +5316,369 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>348</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>350</v>
+        <v>404</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>351</v>
+        <v>405</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>613.5</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>352</v>
+        <v>406</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>353</v>
+        <v>407</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>354</v>
+        <v>408</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="C5" s="45" t="n">
+        <v>409</v>
+      </c>
+      <c r="C5" s="47" t="n">
         <v>0.3</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>356</v>
+        <v>410</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>357</v>
+        <v>411</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>358</v>
+        <v>412</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="C6" s="45" t="n">
+        <v>413</v>
+      </c>
+      <c r="C6" s="47" t="n">
         <v>0.4</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>356</v>
+        <v>410</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>360</v>
+        <v>414</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>358</v>
+        <v>412</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="4" t="s">
-        <v>361</v>
+        <v>415</v>
       </c>
       <c r="C7" s="30" t="n">
         <f aca="false">C4/C5/FX_RMB</f>
         <v>284.027777777778</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>363</v>
+        <v>417</v>
       </c>
       <c r="F7" s="19"/>
       <c r="G7" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
       <c r="B8" s="4" t="s">
-        <v>364</v>
+        <v>418</v>
       </c>
       <c r="C8" s="30" t="n">
         <f aca="false">C4/C6/FX_RMB</f>
         <v>213.020833333333</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>363</v>
+        <v>417</v>
       </c>
       <c r="F8" s="19"/>
       <c r="G8" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
       <c r="B9" s="4" t="s">
-        <v>365</v>
+        <v>419</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">Model!D22</f>
         <v>212.443111513341</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>366</v>
+        <v>420</v>
       </c>
       <c r="F9" s="19"/>
       <c r="G9" s="4" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>367</v>
+        <v>421</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>368</v>
+        <v>422</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>386</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>352</v>
+        <v>406</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>369</v>
+        <v>423</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>370</v>
+        <v>424</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>371</v>
+        <v>425</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="4" t="s">
-        <v>372</v>
+        <v>426</v>
       </c>
       <c r="C11" s="30" t="n">
         <f aca="false">C10/C5/FX_RMB22</f>
         <v>192.039800995025</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>373</v>
+        <v>427</v>
       </c>
       <c r="F11" s="19"/>
       <c r="G11" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="4" t="s">
-        <v>374</v>
+        <v>428</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">Model!C22</f>
         <v>94.052008</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>366</v>
+        <v>420</v>
       </c>
       <c r="F12" s="19"/>
       <c r="G12" s="4" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>375</v>
+        <v>429</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>376</v>
+        <v>430</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>292.7</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>377</v>
+        <v>431</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>378</v>
+        <v>432</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="C14" s="45" t="n">
+        <v>433</v>
+      </c>
+      <c r="C14" s="47" t="n">
         <v>0.25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>356</v>
+        <v>410</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>380</v>
+        <v>434</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>317</v>
+        <v>372</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>381</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
       <c r="B15" s="4" t="s">
-        <v>382</v>
+        <v>436</v>
       </c>
       <c r="C15" s="30" t="n">
         <f aca="false">C13*10/FX_INR/C14</f>
         <v>133.045454545455</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>383</v>
+        <v>437</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="4" t="s">
-        <v>384</v>
+        <v>438</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">Model!D21</f>
         <v>42.728125</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>362</v>
+        <v>416</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>385</v>
+        <v>439</v>
       </c>
       <c r="F16" s="19"/>
       <c r="G16" s="4" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>386</v>
+        <v>440</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>387</v>
+        <v>441</v>
       </c>
       <c r="C17" s="32" t="n">
         <f aca="false">'Feed index'!B5</f>
         <v>1187.7</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>388</v>
+        <v>442</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>389</v>
+        <v>443</v>
       </c>
       <c r="F17" s="19"/>
       <c r="G17" s="4" t="s">
-        <v>390</v>
+        <v>444</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
       <c r="B18" s="4" t="s">
-        <v>391</v>
+        <v>445</v>
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">Model!B7/C17</f>
         <v>4.20981729392944</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>392</v>
+        <v>446</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>393</v>
+        <v>447</v>
       </c>
       <c r="F18" s="19"/>
       <c r="G18" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="4" t="s">
-        <v>394</v>
+        <v>448</v>
       </c>
       <c r="C19" s="30" t="n">
         <f aca="false">C18*500</f>
         <v>2104.90864696472</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>395</v>
+        <v>449</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>396</v>
+        <v>450</v>
       </c>
       <c r="F19" s="19"/>
       <c r="G19" s="4" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>397</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -5086,308 +5719,308 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>398</v>
+        <v>452</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>399</v>
+        <v>453</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>400</v>
+        <v>454</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>401</v>
+        <v>455</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>402</v>
+        <v>456</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>403</v>
+        <v>457</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>404</v>
+        <v>458</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>405</v>
+        <v>459</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>406</v>
+        <v>460</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>407</v>
+        <v>461</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>408</v>
-      </c>
-      <c r="C4" s="46" t="n">
+        <v>462</v>
+      </c>
+      <c r="C4" s="48" t="n">
         <v>6.9</v>
       </c>
-      <c r="D4" s="41" t="n">
+      <c r="D4" s="43" t="n">
         <v>23944</v>
       </c>
-      <c r="E4" s="47" t="n">
+      <c r="E4" s="49" t="n">
         <f aca="false">IF(D4=0,0,C4*1000000/D4)</f>
         <v>288.172402271968</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>411</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>407</v>
+        <v>461</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="C5" s="46" t="n">
+        <v>466</v>
+      </c>
+      <c r="C5" s="48" t="n">
         <v>11.03</v>
       </c>
-      <c r="D5" s="41" t="n">
+      <c r="D5" s="43" t="n">
         <v>18433</v>
       </c>
-      <c r="E5" s="47" t="n">
+      <c r="E5" s="49" t="n">
         <f aca="false">IF(D5=0,0,C5*1000000/D5)</f>
         <v>598.383334237509</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>411</v>
+        <v>465</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>407</v>
+        <v>461</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="C6" s="46" t="n">
+        <v>467</v>
+      </c>
+      <c r="C6" s="48" t="n">
         <v>16.67</v>
       </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="43" t="n">
         <v>212562</v>
       </c>
-      <c r="E6" s="47" t="n">
+      <c r="E6" s="49" t="n">
         <f aca="false">IF(D6=0,0,C6*1000000/D6)</f>
         <v>78.4241774164714</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>411</v>
+        <v>465</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>414</v>
+        <v>468</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>408</v>
-      </c>
-      <c r="C7" s="46" t="n">
+        <v>462</v>
+      </c>
+      <c r="C7" s="48" t="n">
         <v>17.63</v>
       </c>
-      <c r="D7" s="41" t="n">
+      <c r="D7" s="43" t="n">
         <v>114306</v>
       </c>
-      <c r="E7" s="47" t="n">
+      <c r="E7" s="49" t="n">
         <f aca="false">IF(D7=0,0,C7*1000000/D7)</f>
         <v>154.23512326562</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>415</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>414</v>
+        <v>468</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="C8" s="46" t="n">
+        <v>466</v>
+      </c>
+      <c r="C8" s="48" t="n">
         <v>16.97</v>
       </c>
-      <c r="D8" s="41" t="n">
+      <c r="D8" s="43" t="n">
         <v>106865</v>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E8" s="49" t="n">
         <f aca="false">IF(D8=0,0,C8*1000000/D8)</f>
         <v>158.798484068685</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>415</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>414</v>
+        <v>468</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="C9" s="46" t="n">
+        <v>467</v>
+      </c>
+      <c r="C9" s="48" t="n">
         <v>29.95</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="43" t="n">
         <v>201222</v>
       </c>
-      <c r="E9" s="47" t="n">
+      <c r="E9" s="49" t="n">
         <f aca="false">IF(D9=0,0,C9*1000000/D9)</f>
         <v>148.840584031567</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>415</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>416</v>
+        <v>470</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C10" s="46" t="n">
+        <v>95</v>
+      </c>
+      <c r="C10" s="48" t="n">
         <v>11.26287</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="43" t="n">
         <v>203950</v>
       </c>
-      <c r="E10" s="47" t="n">
+      <c r="E10" s="49" t="n">
         <f aca="false">IF(D10=0,0,C10*1000000/D10)</f>
         <v>55.2236822750674</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>417</v>
+        <v>471</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>418</v>
+        <v>472</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>416</v>
+        <v>470</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C11" s="46" t="n">
+        <v>201</v>
+      </c>
+      <c r="C11" s="48" t="n">
         <v>17.394553</v>
       </c>
-      <c r="D11" s="41" t="n">
+      <c r="D11" s="43" t="n">
         <v>136778</v>
       </c>
-      <c r="E11" s="47" t="n">
+      <c r="E11" s="49" t="n">
         <f aca="false">IF(D11=0,0,C11*1000000/D11)</f>
         <v>127.173617102166</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>417</v>
+        <v>471</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>418</v>
+        <v>472</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>416</v>
+        <v>470</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="C12" s="46" t="n">
+        <v>211</v>
+      </c>
+      <c r="C12" s="48" t="n">
         <v>14.755015</v>
       </c>
-      <c r="D12" s="41" t="n">
+      <c r="D12" s="43" t="n">
         <v>343852</v>
       </c>
-      <c r="E12" s="47" t="n">
+      <c r="E12" s="49" t="n">
         <f aca="false">IF(D12=0,0,C12*1000000/D12)</f>
         <v>42.9109471516815</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>417</v>
+        <v>471</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>418</v>
+        <v>472</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>416</v>
+        <v>470</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>420</v>
-      </c>
-      <c r="C13" s="46" t="n">
+        <v>474</v>
+      </c>
+      <c r="C13" s="48" t="n">
         <v>11.742568</v>
       </c>
-      <c r="D13" s="41" t="n">
+      <c r="D13" s="43" t="n">
         <v>206236</v>
       </c>
-      <c r="E13" s="47" t="n">
+      <c r="E13" s="49" t="n">
         <f aca="false">IF(D13=0,0,C13*1000000/D13)</f>
         <v>56.9375278806804</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>417</v>
+        <v>471</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>418</v>
+        <v>472</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>421</v>
+        <v>475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove broker sources from vitamin D3 market-size model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBem8iwrXopPNAx2BvshQ4
</commit_message>
<xml_diff>
--- a/reports/Vitamin D3 market size model.xlsx
+++ b/reports/Vitamin D3 market size model.xlsx
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="461">
   <si>
     <t xml:space="preserve">Vitamin D3 global market size: extrapolation model (2020/2022 base to 2026E)</t>
   </si>
@@ -316,7 +316,7 @@
     <t xml:space="preserve">% of t</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyst assumption. Evidence: FEFAC factsheet (75% of D3 to feed, i.e. 25% non-feed); CITIC via Hubei Gongtong SZSE reply (20.6%, 2021, broker); Garden 2010 legal opinion (19%); Jiemian 2020 (~11%)</t>
+    <t xml:space="preserve">Analyst assumption. Evidence: FEFAC factsheet (75% of D3 to feed, i.e. 25% non-feed); Garden 2010 IPO legal opinion (19%); Jiemian 2020 (~11%)</t>
   </si>
   <si>
     <t xml:space="preserve">2025 (FEFAC)</t>
@@ -1006,7 +1006,7 @@
     <t xml:space="preserve">IFEEDER capacity, t pure D3</t>
   </si>
   <si>
-    <t xml:space="preserve">Compare ~184 t pure in Chinese broker capacity tables (14,740 t D3-500)</t>
+    <t xml:space="preserve">Compare ~183 t pure: 2020 global capacity of 14,600 t D3-500 in Garden CB prospectus p.1-1-375 (Boyar)</t>
   </si>
   <si>
     <t xml:space="preserve">IFEEDER capacity ÷ demand (x)</t>
@@ -1015,7 +1015,7 @@
     <t xml:space="preserve">Basis-independent; FEFAC 2025 says 'five times'</t>
   </si>
   <si>
-    <t xml:space="preserve">Reading: on 500,000 IU/g the IFEEDER supply is ~45 t pure, about 40% below the Boyar-based 2023 path and half the ~100 t pure in dsm-firmenich authors' OPRD paper; on 1,000,000 IU/g it is ~91 t pure (consistent with both), but its capacity would then be ~475 t pure, ~2.6x Chinese capacity tables. No single basis reconciles all three IFEEDER numbers, so it brackets the base case rather than replacing it.</t>
+    <t xml:space="preserve">Reading: on 500,000 IU/g the IFEEDER supply is ~45 t pure, about 40% below the Boyar-based 2023 path and half the ~100 t pure in dsm-firmenich authors' OPRD paper; on 1,000,000 IU/g it is ~91 t pure (consistent with both), but its capacity would then be ~475 t pure, ~2.6x the 2020 capacity in Garden's prospectus (14,600 t = ~183 t pure). No single basis reconciles all three IFEEDER numbers, so it brackets the base case rather than replacing it.</t>
   </si>
   <si>
     <t xml:space="preserve">2026E total value (USD m): feed-grade price x human share</t>
@@ -1156,7 +1156,7 @@
     <t xml:space="preserve">Company filing (management estimate, unsourced)</t>
   </si>
   <si>
-    <t xml:space="preserve">Matches broker demand estimates rather than actual output; Q2 FY22 call (17 Nov 2021) calls it the animal-feed market.</t>
+    <t xml:space="preserve">Well above actual output, so it reads as demand or capacity rather than output; Q2 FY22 call (17 Nov 2021) calls it the animal-feed market.</t>
   </si>
   <si>
     <t xml:space="preserve">Undated</t>
@@ -1204,24 +1204,6 @@
     <t xml:space="preserve">Basis unstated; see Model rows 38-56 for both readings. p.2 table labels 3,639 as capacity.</t>
   </si>
   <si>
-    <t xml:space="preserve">10,308 t (feed 8,189 t)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hubei Gongtong reply to SZSE inquiry, citing CITIC Securities</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 Aug 2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Company filing relaying broker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broker-derived demand.</t>
-  </si>
-  <si>
     <t xml:space="preserve">2021-22</t>
   </si>
   <si>
@@ -1238,33 +1220,6 @@
   </si>
   <si>
     <t xml:space="preserve">Need, not consumption.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demand ~6,750 t; capacity ~14,600 t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demand</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BP Equities, Fermenta Biotech initiating coverage (citing Boyar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mar 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://s3.ap-south-1.amazonaws.com/bpwealth-cdn/pdf/1618577883-BP%20Equities_%20Fermenta%20Biotech%20Ltd._Initiating%20Coverage_BUY_Trgt%20402.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broker research</t>
-  </si>
-  <si>
-    <t xml:space="preserve">English fallback only (broker).</t>
   </si>
   <si>
     <t xml:space="preserve">6,281 t (derived)</t>
@@ -1493,13 +1448,13 @@
     <t xml:space="preserve">Fermenta Annual Report 2025-26, MD&amp;A p.14</t>
   </si>
   <si>
-    <t xml:space="preserve">Fermenta share of human D3 (claim)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BP Equities initiation (broker), Mar 2021: ~25% of human-grade D3 API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broker research (management claim)</t>
+    <t xml:space="preserve">Fermenta share of human D3 (assumption)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst assumption: Fermenta FY26 AR calls itself 'one of the world's three largest manufacturers of pharmaceutical-grade Vitamin D3'; no public share figure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst assumption (company filing)</t>
   </si>
   <si>
     <t xml:space="preserve">Implied human market, as-sold, USD m</t>
@@ -2555,7 +2510,7 @@
       </c>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>55</v>
       </c>
@@ -4649,7 +4604,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -4984,37 +4939,41 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>198</v>
+        <v>354</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>309</v>
       </c>
       <c r="E10" s="44" t="n">
-        <v>10308</v>
+        <v>14793</v>
       </c>
       <c r="F10" s="45" t="n">
         <f aca="false">E10/Potency</f>
-        <v>128.85</v>
+        <v>184.9125</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>310</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="I10" s="3"/>
+        <v>357</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>358</v>
+      </c>
       <c r="J10" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="K10" s="12"/>
+        <v>42</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>44</v>
+      </c>
       <c r="L10" s="3" t="s">
-        <v>358</v>
+        <v>54</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>317</v>
@@ -5023,46 +4982,41 @@
         <v>359</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>361</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>362</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="E11" s="44" t="n">
-        <v>14793</v>
+      <c r="E11" s="46" t="n">
+        <f aca="false">Model!C9</f>
+        <v>6281.017</v>
       </c>
       <c r="F11" s="45" t="n">
         <f aca="false">E11/Potency</f>
-        <v>184.9125</v>
+        <v>78.5127125</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>310</v>
+        <v>362</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="K11" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>54</v>
-      </c>
       <c r="M11" s="3" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="N11" s="12" t="s">
         <v>365</v>
@@ -5070,101 +5024,92 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="E12" s="44" t="n">
-        <v>6750</v>
-      </c>
-      <c r="F12" s="45" t="n">
-        <f aca="false">E12/Potency</f>
-        <v>84.375</v>
-      </c>
+      <c r="E12" s="46"/>
+      <c r="F12" s="3"/>
       <c r="G12" s="3" t="s">
         <v>322</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>369</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="3"/>
+      <c r="J12" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="K12" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="L12" s="3" t="s">
         <v>371</v>
-      </c>
-      <c r="K12" s="13" t="s">
-        <v>372</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>373</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>317</v>
       </c>
       <c r="N12" s="12" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>201</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="E13" s="46"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="K13" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="E13" s="46" t="n">
-        <f aca="false">Model!C9</f>
-        <v>6281.017</v>
-      </c>
-      <c r="F13" s="45" t="n">
-        <f aca="false">E13/Potency</f>
-        <v>78.5127125</v>
-      </c>
-      <c r="G13" s="3" t="s">
+      <c r="L13" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="N13" s="12" t="s">
         <v>377</v>
       </c>
-      <c r="H13" s="12" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="M13" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="N13" s="12" t="s">
+      <c r="C14" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>380</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>383</v>
       </c>
       <c r="E14" s="46"/>
       <c r="F14" s="3"/>
@@ -5172,106 +5117,30 @@
         <v>322</v>
       </c>
       <c r="H14" s="12" t="s">
+        <v>381</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="K14" s="13" t="s">
         <v>384</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="K14" s="13" t="s">
+      <c r="L14" s="3" t="s">
         <v>385</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>386</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>317</v>
       </c>
       <c r="N14" s="12" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="19" t="s">
         <v>387</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="E15" s="46"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>391</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="N15" s="12" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="E16" s="46"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>399</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="M16" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="N16" s="12" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -5282,11 +5151,10 @@
     <hyperlink ref="K7" r:id="rId4" display="https://www.bseindia.com/xml-data/corpfiling/AttachHis/9e5e419e-6095-47a2-a06e-bf49cfe9a712.pdf"/>
     <hyperlink ref="K8" r:id="rId5" display="https://doi.org/10.1021/acs.oprd.4c00333"/>
     <hyperlink ref="K9" r:id="rId6" display="https://www.afia.org/pub/?id=c9faec10-dada-d077-7081-0e9bd8e1bcee"/>
-    <hyperlink ref="K11" r:id="rId7" display="http://static.cninfo.com.cn/finalpage/2023-03-02/1216024789.PDF"/>
-    <hyperlink ref="K12" r:id="rId8" display="https://s3.ap-south-1.amazonaws.com/bpwealth-cdn/pdf/1618577883-BP%20Equities_%20Fermenta%20Biotech%20Ltd._Initiating%20Coverage_BUY_Trgt%20402.pdf"/>
-    <hyperlink ref="K14" r:id="rId9" display="https://ipsnews.net/business/?p=62618"/>
-    <hyperlink ref="K15" r:id="rId10" display="https://www.marketsandmarkets.com/PressReleases/vitamin-d.asp"/>
-    <hyperlink ref="K16" r:id="rId11" display="http://publications.europa.eu/resource/celex/32003D0002"/>
+    <hyperlink ref="K10" r:id="rId7" display="http://static.cninfo.com.cn/finalpage/2023-03-02/1216024789.PDF"/>
+    <hyperlink ref="K12" r:id="rId8" display="https://ipsnews.net/business/?p=62618"/>
+    <hyperlink ref="K13" r:id="rId9" display="https://www.marketsandmarkets.com/PressReleases/vitamin-d.asp"/>
+    <hyperlink ref="K14" r:id="rId10" display="http://publications.europa.eu/resource/celex/32003D0002"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5316,7 +5184,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>403</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5327,7 +5195,7 @@
         <v>27</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>31</v>
@@ -5344,22 +5212,22 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>404</v>
+        <v>389</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>405</v>
+        <v>390</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>613.5</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>406</v>
+        <v>391</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>407</v>
+        <v>392</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>408</v>
+        <v>393</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>54</v>
@@ -5368,19 +5236,19 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2"/>
       <c r="B5" s="4" t="s">
-        <v>409</v>
+        <v>394</v>
       </c>
       <c r="C5" s="47" t="n">
         <v>0.3</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>411</v>
+        <v>396</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>412</v>
+        <v>397</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>54</v>
@@ -5389,19 +5257,19 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2"/>
       <c r="B6" s="4" t="s">
-        <v>413</v>
+        <v>398</v>
       </c>
       <c r="C6" s="47" t="n">
         <v>0.4</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>414</v>
+        <v>399</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>412</v>
+        <v>397</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>54</v>
@@ -5410,141 +5278,141 @@
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2"/>
       <c r="B7" s="4" t="s">
-        <v>415</v>
+        <v>400</v>
       </c>
       <c r="C7" s="30" t="n">
         <f aca="false">C4/C5/FX_RMB</f>
         <v>284.027777777778</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="F7" s="19"/>
       <c r="G7" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
       <c r="B8" s="4" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="C8" s="30" t="n">
         <f aca="false">C4/C6/FX_RMB</f>
         <v>213.020833333333</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="F8" s="19"/>
       <c r="G8" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2"/>
       <c r="B9" s="4" t="s">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">Model!D22</f>
         <v>212.443111513341</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="F9" s="19"/>
       <c r="G9" s="4" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>386</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>406</v>
+        <v>391</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>424</v>
+        <v>409</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>425</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="4" t="s">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="C11" s="30" t="n">
         <f aca="false">C10/C5/FX_RMB22</f>
         <v>192.039800995025</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="F11" s="19"/>
       <c r="G11" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="4" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">Model!C22</f>
         <v>94.052008</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="F12" s="19"/>
       <c r="G12" s="4" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>430</v>
+        <v>415</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>292.7</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>431</v>
+        <v>416</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>432</v>
+        <v>417</v>
       </c>
       <c r="F13" s="23" t="s">
         <v>85</v>
@@ -5553,132 +5421,132 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="4" t="s">
-        <v>433</v>
+        <v>418</v>
       </c>
       <c r="C14" s="47" t="n">
         <v>0.25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>410</v>
+        <v>395</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>434</v>
+        <v>419</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>372</v>
+        <v>85</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>435</v>
+        <v>420</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2"/>
       <c r="B15" s="4" t="s">
-        <v>436</v>
+        <v>421</v>
       </c>
       <c r="C15" s="30" t="n">
         <f aca="false">C13*10/FX_INR/C14</f>
         <v>133.045454545455</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>437</v>
+        <v>422</v>
       </c>
       <c r="F15" s="19"/>
       <c r="G15" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
       <c r="B16" s="4" t="s">
-        <v>438</v>
+        <v>423</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">Model!D21</f>
         <v>42.728125</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>416</v>
+        <v>401</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>439</v>
+        <v>424</v>
       </c>
       <c r="F16" s="19"/>
       <c r="G16" s="4" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>441</v>
+        <v>426</v>
       </c>
       <c r="C17" s="32" t="n">
         <f aca="false">'Feed index'!B5</f>
         <v>1187.7</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>442</v>
+        <v>427</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>443</v>
+        <v>428</v>
       </c>
       <c r="F17" s="19"/>
       <c r="G17" s="4" t="s">
-        <v>444</v>
+        <v>429</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2"/>
       <c r="B18" s="4" t="s">
-        <v>445</v>
+        <v>430</v>
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">Model!B7/C17</f>
         <v>4.20981729392944</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>446</v>
+        <v>431</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>447</v>
+        <v>432</v>
       </c>
       <c r="F18" s="19"/>
       <c r="G18" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2"/>
       <c r="B19" s="4" t="s">
-        <v>448</v>
+        <v>433</v>
       </c>
       <c r="C19" s="30" t="n">
         <f aca="false">C18*500</f>
         <v>2104.90864696472</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>449</v>
+        <v>434</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="F19" s="19"/>
       <c r="G19" s="4" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>451</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>
@@ -5688,7 +5556,7 @@
     <hyperlink ref="F6" r:id="rId3" display="http://static.cninfo.com.cn/finalpage/2025-04-07/1223021870.PDF"/>
     <hyperlink ref="F10" r:id="rId4" display="https://www.lhratings.com/reports/B0648-P66511-2022-GZ2024.pdf"/>
     <hyperlink ref="F13" r:id="rId5" display="https://fermentabiotech.com/wp-content/uploads/2026/09/Annual-Report-2025-26-1.pdf"/>
-    <hyperlink ref="F14" r:id="rId6" display="https://s3.ap-south-1.amazonaws.com/bpwealth-cdn/pdf/1618577883-BP%20Equities_%20Fermenta%20Biotech%20Ltd._Initiating%20Coverage_BUY_Trgt%20402.pdf"/>
+    <hyperlink ref="F14" r:id="rId6" display="https://fermentabiotech.com/wp-content/uploads/2026/09/Annual-Report-2025-26-1.pdf"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5719,41 +5587,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>452</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>453</v>
+        <v>438</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>454</v>
+        <v>439</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>455</v>
+        <v>440</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>457</v>
+        <v>442</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>458</v>
+        <v>443</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>459</v>
+        <v>444</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>460</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>462</v>
+        <v>447</v>
       </c>
       <c r="C4" s="48" t="n">
         <v>6.9</v>
@@ -5766,21 +5634,21 @@
         <v>288.172402271968</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>465</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>466</v>
+        <v>451</v>
       </c>
       <c r="C5" s="48" t="n">
         <v>11.03</v>
@@ -5793,21 +5661,21 @@
         <v>598.383334237509</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>465</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>467</v>
+        <v>452</v>
       </c>
       <c r="C6" s="48" t="n">
         <v>16.67</v>
@@ -5820,21 +5688,21 @@
         <v>78.4241774164714</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>465</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>462</v>
+        <v>447</v>
       </c>
       <c r="C7" s="48" t="n">
         <v>17.63</v>
@@ -5847,21 +5715,21 @@
         <v>154.23512326562</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>466</v>
+        <v>451</v>
       </c>
       <c r="C8" s="48" t="n">
         <v>16.97</v>
@@ -5874,21 +5742,21 @@
         <v>158.798484068685</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>467</v>
+        <v>452</v>
       </c>
       <c r="C9" s="48" t="n">
         <v>29.95</v>
@@ -5901,18 +5769,18 @@
         <v>148.840584031567</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>95</v>
@@ -5928,18 +5796,18 @@
         <v>55.2236822750674</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>201</v>
@@ -5955,18 +5823,18 @@
         <v>127.173617102166</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>211</v>
@@ -5982,21 +5850,21 @@
         <v>42.9109471516815</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>474</v>
+        <v>459</v>
       </c>
       <c r="C13" s="48" t="n">
         <v>11.742568</v>
@@ -6009,18 +5877,18 @@
         <v>56.9375278806804</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>475</v>
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>